<commit_message>
Restore and enhance feed allocation coloring in the program
Update the SheetView component to reintroduce the light green background for the SILO column and implement phase-based background coloring for the FEED ALLOC column based on cumulative feed usage against defined allocation thresholds.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: bf8f1c43-00ef-439e-9e9f-127cf3404bfa
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: b40b9f6b-ed68-4c9b-b384-9a443c2c9238
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/9fb187d0-5a71-40d4-a291-96ab5e107c04/bf8f1c43-00ef-439e-9e9f-127cf3404bfa/mjo8DGh
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/artifacts/feed-program/public/feed-program.xlsx
+++ b/artifacts/feed-program/public/feed-program.xlsx
@@ -3366,9 +3366,6 @@
     <row r="10" hidden="1" ht="15" customHeight="1"/>
     <row r="11" ht="23.25" customHeight="1"/>
     <row r="12" ht="23.25" customHeight="1">
-      <c r="D12">
-        <v>0</v>
-      </c>
       <c r="G12" s="1">
         <f>H2</f>
         <v>26260</v>
@@ -3381,18 +3378,7 @@
         <v>0</v>
       </c>
       <c r="J12">
-        <v>0</v>
-      </c>
-      <c r="K12">
-        <v>0</v>
-      </c>
-      <c r="L12">
-        <v>0</v>
-      </c>
-      <c r="M12">
-        <v>0</v>
-      </c>
-      <c r="O12">
+        <f>(K12+M12+L12)</f>
         <v>0</v>
       </c>
     </row>
@@ -3437,7 +3423,7 @@
       <c r="M13">
         <v>0</v>
       </c>
-      <c r="O13">
+      <c r="O13" s="1">
         <v>0</v>
       </c>
     </row>
@@ -3477,7 +3463,7 @@
       <c r="M14">
         <v>0</v>
       </c>
-      <c r="O14">
+      <c r="O14" s="1">
         <v>0</v>
       </c>
       <c r="R14" s="1">
@@ -3521,7 +3507,7 @@
       <c r="M15">
         <v>0</v>
       </c>
-      <c r="O15">
+      <c r="O15" s="1">
         <v>0</v>
       </c>
       <c r="R15" s="1">
@@ -3565,7 +3551,7 @@
       <c r="M16">
         <v>0</v>
       </c>
-      <c r="O16">
+      <c r="O16" s="1">
         <v>0</v>
       </c>
       <c r="R16" s="1">
@@ -3609,7 +3595,7 @@
       <c r="M17">
         <v>0</v>
       </c>
-      <c r="O17">
+      <c r="O17" s="1">
         <v>0</v>
       </c>
       <c r="R17" s="1">
@@ -3653,7 +3639,7 @@
       <c r="M18">
         <v>0</v>
       </c>
-      <c r="O18">
+      <c r="O18" s="1">
         <v>0</v>
       </c>
       <c r="R18" s="1">
@@ -3700,7 +3686,7 @@
       <c r="M19">
         <v>0</v>
       </c>
-      <c r="O19">
+      <c r="O19" s="1">
         <v>0</v>
       </c>
       <c r="R19" s="1">
@@ -3743,7 +3729,7 @@
       <c r="M20">
         <v>0</v>
       </c>
-      <c r="O20">
+      <c r="O20" s="1">
         <v>0</v>
       </c>
       <c r="R20" s="1">
@@ -3787,7 +3773,7 @@
       <c r="M21">
         <v>0</v>
       </c>
-      <c r="O21">
+      <c r="O21" s="1">
         <v>0</v>
       </c>
       <c r="R21" s="1">
@@ -3833,7 +3819,7 @@
       <c r="M22">
         <v>0</v>
       </c>
-      <c r="O22">
+      <c r="O22" s="1">
         <v>0</v>
       </c>
       <c r="R22" s="1">
@@ -3877,7 +3863,7 @@
       <c r="M23">
         <v>0</v>
       </c>
-      <c r="O23">
+      <c r="O23" s="1">
         <v>0</v>
       </c>
       <c r="R23" s="1">
@@ -3921,7 +3907,7 @@
       <c r="M24">
         <v>0</v>
       </c>
-      <c r="O24">
+      <c r="O24" s="1">
         <v>0</v>
       </c>
       <c r="R24" s="1">
@@ -3965,7 +3951,7 @@
       <c r="M25">
         <v>0</v>
       </c>
-      <c r="O25">
+      <c r="O25" s="1">
         <v>0</v>
       </c>
       <c r="R25" s="1">
@@ -4012,7 +3998,7 @@
       <c r="M26">
         <v>0</v>
       </c>
-      <c r="O26">
+      <c r="O26" s="1">
         <v>0</v>
       </c>
       <c r="R26" s="1">
@@ -4056,7 +4042,7 @@
       <c r="M27">
         <v>0</v>
       </c>
-      <c r="O27">
+      <c r="O27" s="1">
         <v>0</v>
       </c>
       <c r="R27" s="1">
@@ -4100,7 +4086,7 @@
       <c r="M28">
         <v>0</v>
       </c>
-      <c r="O28">
+      <c r="O28" s="1">
         <v>0</v>
       </c>
       <c r="R28" s="1">
@@ -4147,7 +4133,7 @@
       <c r="M29">
         <v>0</v>
       </c>
-      <c r="O29">
+      <c r="O29" s="1">
         <v>0</v>
       </c>
       <c r="R29" s="1">
@@ -4191,7 +4177,7 @@
       <c r="M30">
         <v>0</v>
       </c>
-      <c r="O30">
+      <c r="O30" s="1">
         <v>0</v>
       </c>
       <c r="R30" s="1">
@@ -4235,7 +4221,7 @@
       <c r="M31">
         <v>0</v>
       </c>
-      <c r="O31">
+      <c r="O31" s="1">
         <v>0</v>
       </c>
       <c r="R31" s="1">
@@ -4279,7 +4265,7 @@
       <c r="M32">
         <v>0</v>
       </c>
-      <c r="O32">
+      <c r="O32" s="1">
         <v>0</v>
       </c>
       <c r="R32" s="1">
@@ -4326,7 +4312,7 @@
       <c r="M33">
         <v>0</v>
       </c>
-      <c r="O33">
+      <c r="O33" s="1">
         <v>0</v>
       </c>
       <c r="R33" s="1">
@@ -4370,7 +4356,7 @@
       <c r="M34">
         <v>0</v>
       </c>
-      <c r="O34">
+      <c r="O34" s="1">
         <v>0</v>
       </c>
       <c r="R34" s="1">
@@ -4414,7 +4400,7 @@
       <c r="M35">
         <v>0</v>
       </c>
-      <c r="O35">
+      <c r="O35" s="1">
         <v>0</v>
       </c>
       <c r="R35" s="1">
@@ -4461,7 +4447,7 @@
       <c r="M36">
         <v>0</v>
       </c>
-      <c r="O36">
+      <c r="O36" s="1">
         <v>0</v>
       </c>
       <c r="R36" s="1">
@@ -4505,7 +4491,7 @@
       <c r="M37">
         <v>0</v>
       </c>
-      <c r="O37">
+      <c r="O37" s="1">
         <v>0</v>
       </c>
       <c r="R37" s="1">
@@ -4549,7 +4535,7 @@
       <c r="M38">
         <v>0</v>
       </c>
-      <c r="O38">
+      <c r="O38" s="1">
         <v>0</v>
       </c>
       <c r="R38" s="1">
@@ -4593,7 +4579,7 @@
       <c r="M39">
         <v>0</v>
       </c>
-      <c r="O39">
+      <c r="O39" s="1">
         <v>0</v>
       </c>
       <c r="R39" s="1">
@@ -4637,7 +4623,7 @@
       <c r="M40">
         <v>0</v>
       </c>
-      <c r="O40">
+      <c r="O40" s="1">
         <v>0</v>
       </c>
       <c r="R40" s="1">
@@ -4681,7 +4667,7 @@
       <c r="M41">
         <v>0</v>
       </c>
-      <c r="O41">
+      <c r="O41" s="1">
         <v>0</v>
       </c>
       <c r="R41" s="1">
@@ -4725,7 +4711,7 @@
       <c r="M42">
         <v>0</v>
       </c>
-      <c r="O42">
+      <c r="O42" s="1">
         <v>0</v>
       </c>
       <c r="R42" s="1">
@@ -4769,7 +4755,7 @@
       <c r="M43">
         <v>0</v>
       </c>
-      <c r="O43">
+      <c r="O43" s="1">
         <v>0</v>
       </c>
       <c r="R43" s="1">
@@ -4813,7 +4799,7 @@
       <c r="M44">
         <v>0</v>
       </c>
-      <c r="O44">
+      <c r="O44" s="1">
         <v>0</v>
       </c>
       <c r="R44" s="1">
@@ -4856,7 +4842,7 @@
       <c r="M45">
         <v>0</v>
       </c>
-      <c r="O45">
+      <c r="O45" s="1">
         <v>0</v>
       </c>
       <c r="R45" s="1">
@@ -4899,7 +4885,7 @@
       <c r="M46">
         <v>0</v>
       </c>
-      <c r="O46">
+      <c r="O46" s="1">
         <v>0</v>
       </c>
       <c r="R46" s="1">
@@ -4942,7 +4928,7 @@
       <c r="M47">
         <v>0</v>
       </c>
-      <c r="O47">
+      <c r="O47" s="1">
         <v>0</v>
       </c>
       <c r="R47" s="1">
@@ -4985,7 +4971,7 @@
       <c r="M48">
         <v>0</v>
       </c>
-      <c r="O48">
+      <c r="O48" s="1">
         <v>0</v>
       </c>
       <c r="R48" s="1">
@@ -5028,7 +5014,7 @@
       <c r="M49">
         <v>0</v>
       </c>
-      <c r="O49">
+      <c r="O49" s="1">
         <v>0</v>
       </c>
       <c r="R49" s="1">
@@ -5071,7 +5057,7 @@
       <c r="M50">
         <v>0</v>
       </c>
-      <c r="O50">
+      <c r="O50" s="1">
         <v>0</v>
       </c>
       <c r="R50" s="1">
@@ -5114,7 +5100,7 @@
       <c r="M51">
         <v>0</v>
       </c>
-      <c r="O51">
+      <c r="O51" s="1">
         <v>0</v>
       </c>
       <c r="R51" s="1">
@@ -5157,7 +5143,7 @@
       <c r="M52">
         <v>0</v>
       </c>
-      <c r="O52">
+      <c r="O52" s="1">
         <v>0</v>
       </c>
       <c r="R52" s="1">
@@ -5200,7 +5186,7 @@
       <c r="M53">
         <v>0</v>
       </c>
-      <c r="O53">
+      <c r="O53" s="1">
         <v>0</v>
       </c>
       <c r="R53" s="1">
@@ -5243,7 +5229,7 @@
       <c r="M54">
         <v>0</v>
       </c>
-      <c r="O54">
+      <c r="O54" s="1">
         <v>0</v>
       </c>
       <c r="R54" s="1">
@@ -5286,7 +5272,7 @@
       <c r="M55">
         <v>0</v>
       </c>
-      <c r="O55">
+      <c r="O55" s="1">
         <v>0</v>
       </c>
       <c r="R55" s="1">
@@ -5329,7 +5315,7 @@
       <c r="M56">
         <v>0</v>
       </c>
-      <c r="O56">
+      <c r="O56" s="1">
         <v>0</v>
       </c>
       <c r="R56" s="1">
@@ -5372,7 +5358,7 @@
       <c r="M57">
         <v>0</v>
       </c>
-      <c r="O57">
+      <c r="O57" s="1">
         <v>0</v>
       </c>
       <c r="R57" s="1">
@@ -5415,7 +5401,7 @@
       <c r="M58">
         <v>0</v>
       </c>
-      <c r="O58">
+      <c r="O58" s="1">
         <v>0</v>
       </c>
       <c r="R58" s="1">
@@ -5458,7 +5444,7 @@
       <c r="M59">
         <v>0</v>
       </c>
-      <c r="O59">
+      <c r="O59" s="1">
         <v>0</v>
       </c>
       <c r="R59" s="1">
@@ -5501,7 +5487,7 @@
       <c r="M60">
         <v>0</v>
       </c>
-      <c r="O60">
+      <c r="O60" s="1">
         <v>0</v>
       </c>
       <c r="R60" s="1">
@@ -5544,7 +5530,7 @@
       <c r="M61">
         <v>0</v>
       </c>
-      <c r="O61">
+      <c r="O61" s="1">
         <v>0</v>
       </c>
       <c r="R61" s="1">
@@ -5587,7 +5573,7 @@
       <c r="M62">
         <v>0</v>
       </c>
-      <c r="O62">
+      <c r="O62" s="1">
         <v>0</v>
       </c>
       <c r="R62" s="1">
@@ -5630,7 +5616,7 @@
       <c r="M63">
         <v>0</v>
       </c>
-      <c r="O63">
+      <c r="O63" s="1">
         <v>0</v>
       </c>
       <c r="R63" s="1">
@@ -5673,7 +5659,7 @@
       <c r="M64">
         <v>0</v>
       </c>
-      <c r="O64">
+      <c r="O64" s="1">
         <v>0</v>
       </c>
       <c r="R64" s="1">
@@ -5716,7 +5702,7 @@
       <c r="M65">
         <v>0</v>
       </c>
-      <c r="O65">
+      <c r="O65" s="1">
         <v>0</v>
       </c>
       <c r="R65" s="1">
@@ -5759,7 +5745,7 @@
       <c r="M66">
         <v>0</v>
       </c>
-      <c r="O66">
+      <c r="O66" s="1">
         <v>0</v>
       </c>
       <c r="R66" s="1">
@@ -5802,7 +5788,7 @@
       <c r="M67">
         <v>0</v>
       </c>
-      <c r="O67">
+      <c r="O67" s="1">
         <v>0</v>
       </c>
       <c r="R67" s="1">
@@ -5845,7 +5831,7 @@
       <c r="M68">
         <v>0</v>
       </c>
-      <c r="O68">
+      <c r="O68" s="1">
         <v>0</v>
       </c>
       <c r="R68" s="1">
@@ -5889,7 +5875,7 @@
       <c r="M69">
         <v>0</v>
       </c>
-      <c r="O69">
+      <c r="O69" s="1">
         <v>0</v>
       </c>
       <c r="R69" s="1">
@@ -5933,7 +5919,7 @@
       <c r="M70">
         <v>0</v>
       </c>
-      <c r="O70">
+      <c r="O70" s="1">
         <v>0</v>
       </c>
       <c r="R70" s="1">
@@ -5973,7 +5959,7 @@
       <c r="M71">
         <v>0</v>
       </c>
-      <c r="O71">
+      <c r="O71" s="1">
         <v>0</v>
       </c>
       <c r="R71" s="1">
@@ -6009,7 +5995,7 @@
       <c r="M72">
         <v>0</v>
       </c>
-      <c r="O72">
+      <c r="O72" s="1">
         <v>0</v>
       </c>
       <c r="R72" s="1">
@@ -7345,9 +7331,6 @@
     <row r="10" hidden="1" ht="15" customHeight="1"/>
     <row r="11" ht="23.25" customHeight="1"/>
     <row r="12" ht="23.25" customHeight="1">
-      <c r="D12">
-        <v>0</v>
-      </c>
       <c r="G12" s="1">
         <f>H2</f>
         <v>26000</v>
@@ -7360,18 +7343,7 @@
         <v>0</v>
       </c>
       <c r="J12">
-        <v>0</v>
-      </c>
-      <c r="K12">
-        <v>0</v>
-      </c>
-      <c r="L12">
-        <v>0</v>
-      </c>
-      <c r="M12">
-        <v>0</v>
-      </c>
-      <c r="O12">
+        <f>(K12+M12+L12)</f>
         <v>0</v>
       </c>
     </row>
@@ -7416,7 +7388,7 @@
       <c r="M13">
         <v>0</v>
       </c>
-      <c r="O13">
+      <c r="O13" s="1">
         <v>0</v>
       </c>
     </row>
@@ -7456,7 +7428,7 @@
       <c r="M14">
         <v>0</v>
       </c>
-      <c r="O14">
+      <c r="O14" s="1">
         <v>0</v>
       </c>
       <c r="R14" s="1">
@@ -7500,7 +7472,7 @@
       <c r="M15">
         <v>0</v>
       </c>
-      <c r="O15">
+      <c r="O15" s="1">
         <v>0</v>
       </c>
       <c r="R15" s="1">
@@ -7544,7 +7516,7 @@
       <c r="M16">
         <v>0</v>
       </c>
-      <c r="O16">
+      <c r="O16" s="1">
         <v>0</v>
       </c>
       <c r="R16" s="1">
@@ -7588,7 +7560,7 @@
       <c r="M17">
         <v>0</v>
       </c>
-      <c r="O17">
+      <c r="O17" s="1">
         <v>0</v>
       </c>
       <c r="R17" s="1">
@@ -7632,7 +7604,7 @@
       <c r="M18">
         <v>0</v>
       </c>
-      <c r="O18">
+      <c r="O18" s="1">
         <v>0</v>
       </c>
       <c r="R18" s="1">
@@ -7679,7 +7651,7 @@
       <c r="M19">
         <v>0</v>
       </c>
-      <c r="O19">
+      <c r="O19" s="1">
         <v>0</v>
       </c>
       <c r="R19" s="1">
@@ -7722,7 +7694,7 @@
       <c r="M20">
         <v>0</v>
       </c>
-      <c r="O20">
+      <c r="O20" s="1">
         <v>0</v>
       </c>
       <c r="R20" s="1">
@@ -7766,7 +7738,7 @@
       <c r="M21">
         <v>0</v>
       </c>
-      <c r="O21">
+      <c r="O21" s="1">
         <v>0</v>
       </c>
       <c r="R21" s="1">
@@ -7812,7 +7784,7 @@
       <c r="M22">
         <v>0</v>
       </c>
-      <c r="O22">
+      <c r="O22" s="1">
         <v>0</v>
       </c>
       <c r="R22" s="1">
@@ -7856,7 +7828,7 @@
       <c r="M23">
         <v>0</v>
       </c>
-      <c r="O23">
+      <c r="O23" s="1">
         <v>0</v>
       </c>
       <c r="R23" s="1">
@@ -7900,7 +7872,7 @@
       <c r="M24">
         <v>0</v>
       </c>
-      <c r="O24">
+      <c r="O24" s="1">
         <v>0</v>
       </c>
       <c r="R24" s="1">
@@ -7944,7 +7916,7 @@
       <c r="M25">
         <v>0</v>
       </c>
-      <c r="O25">
+      <c r="O25" s="1">
         <v>0</v>
       </c>
       <c r="R25" s="1">
@@ -7991,7 +7963,7 @@
       <c r="M26">
         <v>0</v>
       </c>
-      <c r="O26">
+      <c r="O26" s="1">
         <v>0</v>
       </c>
       <c r="R26" s="1">
@@ -8035,7 +8007,7 @@
       <c r="M27">
         <v>0</v>
       </c>
-      <c r="O27">
+      <c r="O27" s="1">
         <v>0</v>
       </c>
       <c r="R27" s="1">
@@ -8079,7 +8051,7 @@
       <c r="M28">
         <v>0</v>
       </c>
-      <c r="O28">
+      <c r="O28" s="1">
         <v>0</v>
       </c>
       <c r="R28" s="1">
@@ -8126,7 +8098,7 @@
       <c r="M29">
         <v>0</v>
       </c>
-      <c r="O29">
+      <c r="O29" s="1">
         <v>0</v>
       </c>
       <c r="R29" s="1">
@@ -8170,7 +8142,7 @@
       <c r="M30">
         <v>0</v>
       </c>
-      <c r="O30">
+      <c r="O30" s="1">
         <v>0</v>
       </c>
       <c r="R30" s="1">
@@ -8214,7 +8186,7 @@
       <c r="M31">
         <v>0</v>
       </c>
-      <c r="O31">
+      <c r="O31" s="1">
         <v>0</v>
       </c>
       <c r="R31" s="1">
@@ -8258,7 +8230,7 @@
       <c r="M32">
         <v>0</v>
       </c>
-      <c r="O32">
+      <c r="O32" s="1">
         <v>0</v>
       </c>
       <c r="R32" s="1">
@@ -8305,7 +8277,7 @@
       <c r="M33">
         <v>0</v>
       </c>
-      <c r="O33">
+      <c r="O33" s="1">
         <v>0</v>
       </c>
       <c r="R33" s="1">
@@ -8349,7 +8321,7 @@
       <c r="M34">
         <v>0</v>
       </c>
-      <c r="O34">
+      <c r="O34" s="1">
         <v>0</v>
       </c>
       <c r="R34" s="1">
@@ -8393,7 +8365,7 @@
       <c r="M35">
         <v>0</v>
       </c>
-      <c r="O35">
+      <c r="O35" s="1">
         <v>0</v>
       </c>
       <c r="R35" s="1">
@@ -8440,7 +8412,7 @@
       <c r="M36">
         <v>0</v>
       </c>
-      <c r="O36">
+      <c r="O36" s="1">
         <v>0</v>
       </c>
       <c r="R36" s="1">
@@ -8484,7 +8456,7 @@
       <c r="M37">
         <v>0</v>
       </c>
-      <c r="O37">
+      <c r="O37" s="1">
         <v>0</v>
       </c>
       <c r="R37" s="1">
@@ -8528,7 +8500,7 @@
       <c r="M38">
         <v>0</v>
       </c>
-      <c r="O38">
+      <c r="O38" s="1">
         <v>0</v>
       </c>
       <c r="R38" s="1">
@@ -8572,7 +8544,7 @@
       <c r="M39">
         <v>0</v>
       </c>
-      <c r="O39">
+      <c r="O39" s="1">
         <v>0</v>
       </c>
       <c r="R39" s="1">
@@ -8616,7 +8588,7 @@
       <c r="M40">
         <v>0</v>
       </c>
-      <c r="O40">
+      <c r="O40" s="1">
         <v>0</v>
       </c>
       <c r="R40" s="1">
@@ -8660,7 +8632,7 @@
       <c r="M41">
         <v>0</v>
       </c>
-      <c r="O41">
+      <c r="O41" s="1">
         <v>0</v>
       </c>
       <c r="R41" s="1">
@@ -8704,7 +8676,7 @@
       <c r="M42">
         <v>0</v>
       </c>
-      <c r="O42">
+      <c r="O42" s="1">
         <v>0</v>
       </c>
       <c r="R42" s="1">
@@ -8748,7 +8720,7 @@
       <c r="M43">
         <v>0</v>
       </c>
-      <c r="O43">
+      <c r="O43" s="1">
         <v>0</v>
       </c>
       <c r="R43" s="1">
@@ -8792,7 +8764,7 @@
       <c r="M44">
         <v>0</v>
       </c>
-      <c r="O44">
+      <c r="O44" s="1">
         <v>0</v>
       </c>
       <c r="R44" s="1">
@@ -8835,7 +8807,7 @@
       <c r="M45">
         <v>0</v>
       </c>
-      <c r="O45">
+      <c r="O45" s="1">
         <v>0</v>
       </c>
       <c r="R45" s="1">
@@ -8878,7 +8850,7 @@
       <c r="M46">
         <v>0</v>
       </c>
-      <c r="O46">
+      <c r="O46" s="1">
         <v>0</v>
       </c>
       <c r="R46" s="1">
@@ -8921,7 +8893,7 @@
       <c r="M47">
         <v>0</v>
       </c>
-      <c r="O47">
+      <c r="O47" s="1">
         <v>0</v>
       </c>
       <c r="R47" s="1">
@@ -8964,7 +8936,7 @@
       <c r="M48">
         <v>0</v>
       </c>
-      <c r="O48">
+      <c r="O48" s="1">
         <v>0</v>
       </c>
       <c r="R48" s="1">
@@ -9007,7 +8979,7 @@
       <c r="M49">
         <v>0</v>
       </c>
-      <c r="O49">
+      <c r="O49" s="1">
         <v>0</v>
       </c>
       <c r="R49" s="1">
@@ -9050,7 +9022,7 @@
       <c r="M50">
         <v>0</v>
       </c>
-      <c r="O50">
+      <c r="O50" s="1">
         <v>0</v>
       </c>
       <c r="R50" s="1">
@@ -9093,7 +9065,7 @@
       <c r="M51">
         <v>0</v>
       </c>
-      <c r="O51">
+      <c r="O51" s="1">
         <v>0</v>
       </c>
       <c r="R51" s="1">
@@ -9136,7 +9108,7 @@
       <c r="M52">
         <v>0</v>
       </c>
-      <c r="O52">
+      <c r="O52" s="1">
         <v>0</v>
       </c>
       <c r="R52" s="1">
@@ -9179,7 +9151,7 @@
       <c r="M53">
         <v>0</v>
       </c>
-      <c r="O53">
+      <c r="O53" s="1">
         <v>0</v>
       </c>
       <c r="R53" s="1">
@@ -9222,7 +9194,7 @@
       <c r="M54">
         <v>0</v>
       </c>
-      <c r="O54">
+      <c r="O54" s="1">
         <v>0</v>
       </c>
       <c r="R54" s="1">
@@ -9265,7 +9237,7 @@
       <c r="M55">
         <v>0</v>
       </c>
-      <c r="O55">
+      <c r="O55" s="1">
         <v>0</v>
       </c>
       <c r="R55" s="1">
@@ -9308,7 +9280,7 @@
       <c r="M56">
         <v>0</v>
       </c>
-      <c r="O56">
+      <c r="O56" s="1">
         <v>0</v>
       </c>
       <c r="R56" s="1">
@@ -9351,7 +9323,7 @@
       <c r="M57">
         <v>0</v>
       </c>
-      <c r="O57">
+      <c r="O57" s="1">
         <v>0</v>
       </c>
       <c r="R57" s="1">
@@ -9394,7 +9366,7 @@
       <c r="M58">
         <v>0</v>
       </c>
-      <c r="O58">
+      <c r="O58" s="1">
         <v>0</v>
       </c>
       <c r="R58" s="1">
@@ -9437,7 +9409,7 @@
       <c r="M59">
         <v>0</v>
       </c>
-      <c r="O59">
+      <c r="O59" s="1">
         <v>0</v>
       </c>
       <c r="R59" s="1">
@@ -9480,7 +9452,7 @@
       <c r="M60">
         <v>0</v>
       </c>
-      <c r="O60">
+      <c r="O60" s="1">
         <v>0</v>
       </c>
       <c r="R60" s="1">
@@ -9523,7 +9495,7 @@
       <c r="M61">
         <v>0</v>
       </c>
-      <c r="O61">
+      <c r="O61" s="1">
         <v>0</v>
       </c>
       <c r="R61" s="1">
@@ -9566,7 +9538,7 @@
       <c r="M62">
         <v>0</v>
       </c>
-      <c r="O62">
+      <c r="O62" s="1">
         <v>0</v>
       </c>
       <c r="R62" s="1">
@@ -9609,7 +9581,7 @@
       <c r="M63">
         <v>0</v>
       </c>
-      <c r="O63">
+      <c r="O63" s="1">
         <v>0</v>
       </c>
       <c r="R63" s="1">
@@ -9652,7 +9624,7 @@
       <c r="M64">
         <v>0</v>
       </c>
-      <c r="O64">
+      <c r="O64" s="1">
         <v>0</v>
       </c>
       <c r="R64" s="1">
@@ -9695,7 +9667,7 @@
       <c r="M65">
         <v>0</v>
       </c>
-      <c r="O65">
+      <c r="O65" s="1">
         <v>0</v>
       </c>
       <c r="R65" s="1">
@@ -9738,7 +9710,7 @@
       <c r="M66">
         <v>0</v>
       </c>
-      <c r="O66">
+      <c r="O66" s="1">
         <v>0</v>
       </c>
       <c r="R66" s="1">
@@ -9781,7 +9753,7 @@
       <c r="M67">
         <v>0</v>
       </c>
-      <c r="O67">
+      <c r="O67" s="1">
         <v>0</v>
       </c>
       <c r="R67" s="1">
@@ -9824,7 +9796,7 @@
       <c r="M68">
         <v>0</v>
       </c>
-      <c r="O68">
+      <c r="O68" s="1">
         <v>0</v>
       </c>
       <c r="R68" s="1">
@@ -9868,7 +9840,7 @@
       <c r="M69">
         <v>0</v>
       </c>
-      <c r="O69">
+      <c r="O69" s="1">
         <v>0</v>
       </c>
       <c r="R69" s="1">
@@ -9912,7 +9884,7 @@
       <c r="M70">
         <v>0</v>
       </c>
-      <c r="O70">
+      <c r="O70" s="1">
         <v>0</v>
       </c>
       <c r="R70" s="1">
@@ -9952,7 +9924,7 @@
       <c r="M71">
         <v>0</v>
       </c>
-      <c r="O71">
+      <c r="O71" s="1">
         <v>0</v>
       </c>
       <c r="R71" s="1">
@@ -9988,7 +9960,7 @@
       <c r="M72">
         <v>0</v>
       </c>
-      <c r="O72">
+      <c r="O72" s="1">
         <v>0</v>
       </c>
       <c r="R72" s="1">
@@ -11324,9 +11296,6 @@
     <row r="10" hidden="1" ht="15" customHeight="1"/>
     <row r="11" ht="23.25" customHeight="1"/>
     <row r="12" ht="23.25" customHeight="1">
-      <c r="D12">
-        <v>0</v>
-      </c>
       <c r="G12" s="1">
         <f>H2</f>
         <v>26000</v>
@@ -11339,18 +11308,7 @@
         <v>0</v>
       </c>
       <c r="J12">
-        <v>0</v>
-      </c>
-      <c r="K12">
-        <v>0</v>
-      </c>
-      <c r="L12">
-        <v>0</v>
-      </c>
-      <c r="M12">
-        <v>0</v>
-      </c>
-      <c r="O12">
+        <f>(K12+M12+L12)</f>
         <v>0</v>
       </c>
     </row>
@@ -11395,7 +11353,7 @@
       <c r="M13">
         <v>0</v>
       </c>
-      <c r="O13">
+      <c r="O13" s="1">
         <v>0</v>
       </c>
     </row>
@@ -11435,7 +11393,7 @@
       <c r="M14">
         <v>0</v>
       </c>
-      <c r="O14">
+      <c r="O14" s="1">
         <v>0</v>
       </c>
       <c r="R14" s="1">
@@ -11479,7 +11437,7 @@
       <c r="M15">
         <v>0</v>
       </c>
-      <c r="O15">
+      <c r="O15" s="1">
         <v>0</v>
       </c>
       <c r="R15" s="1">
@@ -11526,7 +11484,7 @@
       <c r="M16">
         <v>0</v>
       </c>
-      <c r="O16">
+      <c r="O16" s="1">
         <v>0</v>
       </c>
       <c r="R16" s="1">
@@ -11570,7 +11528,7 @@
       <c r="M17">
         <v>0</v>
       </c>
-      <c r="O17">
+      <c r="O17" s="1">
         <v>0</v>
       </c>
       <c r="R17" s="1">
@@ -11614,7 +11572,7 @@
       <c r="M18">
         <v>0</v>
       </c>
-      <c r="O18">
+      <c r="O18" s="1">
         <v>0</v>
       </c>
       <c r="R18" s="1">
@@ -11661,7 +11619,7 @@
       <c r="M19">
         <v>0</v>
       </c>
-      <c r="O19">
+      <c r="O19" s="1">
         <v>0</v>
       </c>
       <c r="R19" s="1">
@@ -11704,7 +11662,7 @@
       <c r="M20">
         <v>0</v>
       </c>
-      <c r="O20">
+      <c r="O20" s="1">
         <v>0</v>
       </c>
       <c r="R20" s="1">
@@ -11748,7 +11706,7 @@
       <c r="M21">
         <v>0</v>
       </c>
-      <c r="O21">
+      <c r="O21" s="1">
         <v>0</v>
       </c>
       <c r="R21" s="1">
@@ -11791,7 +11749,7 @@
       <c r="M22">
         <v>0</v>
       </c>
-      <c r="O22">
+      <c r="O22" s="1">
         <v>0</v>
       </c>
       <c r="R22" s="1">
@@ -11838,7 +11796,7 @@
       <c r="M23">
         <v>0</v>
       </c>
-      <c r="O23">
+      <c r="O23" s="1">
         <v>0</v>
       </c>
       <c r="R23" s="1">
@@ -11882,7 +11840,7 @@
       <c r="M24">
         <v>0</v>
       </c>
-      <c r="O24">
+      <c r="O24" s="1">
         <v>0</v>
       </c>
       <c r="R24" s="1">
@@ -11926,7 +11884,7 @@
       <c r="M25">
         <v>0</v>
       </c>
-      <c r="O25">
+      <c r="O25" s="1">
         <v>0</v>
       </c>
       <c r="R25" s="1">
@@ -11973,7 +11931,7 @@
       <c r="M26">
         <v>0</v>
       </c>
-      <c r="O26">
+      <c r="O26" s="1">
         <v>0</v>
       </c>
       <c r="R26" s="1">
@@ -12017,7 +11975,7 @@
       <c r="M27">
         <v>0</v>
       </c>
-      <c r="O27">
+      <c r="O27" s="1">
         <v>0</v>
       </c>
       <c r="R27" s="1">
@@ -12061,7 +12019,7 @@
       <c r="M28">
         <v>0</v>
       </c>
-      <c r="O28">
+      <c r="O28" s="1">
         <v>0</v>
       </c>
       <c r="R28" s="1">
@@ -12105,7 +12063,7 @@
       <c r="M29">
         <v>0</v>
       </c>
-      <c r="O29">
+      <c r="O29" s="1">
         <v>0</v>
       </c>
       <c r="R29" s="1">
@@ -12152,7 +12110,7 @@
       <c r="M30">
         <v>0</v>
       </c>
-      <c r="O30">
+      <c r="O30" s="1">
         <v>0</v>
       </c>
       <c r="R30" s="1">
@@ -12196,7 +12154,7 @@
       <c r="M31">
         <v>0</v>
       </c>
-      <c r="O31">
+      <c r="O31" s="1">
         <v>0</v>
       </c>
       <c r="R31" s="1">
@@ -12240,7 +12198,7 @@
       <c r="M32">
         <v>0</v>
       </c>
-      <c r="O32">
+      <c r="O32" s="1">
         <v>0</v>
       </c>
       <c r="R32" s="1">
@@ -12287,7 +12245,7 @@
       <c r="M33">
         <v>0</v>
       </c>
-      <c r="O33">
+      <c r="O33" s="1">
         <v>0</v>
       </c>
       <c r="R33" s="1">
@@ -12331,7 +12289,7 @@
       <c r="M34">
         <v>0</v>
       </c>
-      <c r="O34">
+      <c r="O34" s="1">
         <v>0</v>
       </c>
       <c r="R34" s="1">
@@ -12375,7 +12333,7 @@
       <c r="M35">
         <v>0</v>
       </c>
-      <c r="O35">
+      <c r="O35" s="1">
         <v>0</v>
       </c>
       <c r="R35" s="1">
@@ -12419,7 +12377,7 @@
       <c r="M36">
         <v>0</v>
       </c>
-      <c r="O36">
+      <c r="O36" s="1">
         <v>0</v>
       </c>
       <c r="R36" s="1">
@@ -12463,7 +12421,7 @@
       <c r="M37">
         <v>0</v>
       </c>
-      <c r="O37">
+      <c r="O37" s="1">
         <v>0</v>
       </c>
       <c r="R37" s="1">
@@ -12507,7 +12465,7 @@
       <c r="M38">
         <v>0</v>
       </c>
-      <c r="O38">
+      <c r="O38" s="1">
         <v>0</v>
       </c>
       <c r="R38" s="1">
@@ -12551,7 +12509,7 @@
       <c r="M39">
         <v>0</v>
       </c>
-      <c r="O39">
+      <c r="O39" s="1">
         <v>0</v>
       </c>
       <c r="R39" s="1">
@@ -12595,7 +12553,7 @@
       <c r="M40">
         <v>0</v>
       </c>
-      <c r="O40">
+      <c r="O40" s="1">
         <v>0</v>
       </c>
       <c r="R40" s="1">
@@ -12639,7 +12597,7 @@
       <c r="M41">
         <v>0</v>
       </c>
-      <c r="O41">
+      <c r="O41" s="1">
         <v>0</v>
       </c>
       <c r="R41" s="1">
@@ -12683,7 +12641,7 @@
       <c r="M42">
         <v>0</v>
       </c>
-      <c r="O42">
+      <c r="O42" s="1">
         <v>0</v>
       </c>
       <c r="R42" s="1">
@@ -12727,7 +12685,7 @@
       <c r="M43">
         <v>0</v>
       </c>
-      <c r="O43">
+      <c r="O43" s="1">
         <v>0</v>
       </c>
       <c r="R43" s="1">
@@ -12771,7 +12729,7 @@
       <c r="M44">
         <v>0</v>
       </c>
-      <c r="O44">
+      <c r="O44" s="1">
         <v>0</v>
       </c>
       <c r="R44" s="1">
@@ -12814,7 +12772,7 @@
       <c r="M45">
         <v>0</v>
       </c>
-      <c r="O45">
+      <c r="O45" s="1">
         <v>0</v>
       </c>
       <c r="R45" s="1">
@@ -12857,7 +12815,7 @@
       <c r="M46">
         <v>0</v>
       </c>
-      <c r="O46">
+      <c r="O46" s="1">
         <v>0</v>
       </c>
       <c r="R46" s="1">
@@ -12900,7 +12858,7 @@
       <c r="M47">
         <v>0</v>
       </c>
-      <c r="O47">
+      <c r="O47" s="1">
         <v>0</v>
       </c>
       <c r="R47" s="1">
@@ -12943,7 +12901,7 @@
       <c r="M48">
         <v>0</v>
       </c>
-      <c r="O48">
+      <c r="O48" s="1">
         <v>0</v>
       </c>
       <c r="R48" s="1">
@@ -12986,7 +12944,7 @@
       <c r="M49">
         <v>0</v>
       </c>
-      <c r="O49">
+      <c r="O49" s="1">
         <v>0</v>
       </c>
       <c r="R49" s="1">
@@ -13029,7 +12987,7 @@
       <c r="M50">
         <v>0</v>
       </c>
-      <c r="O50">
+      <c r="O50" s="1">
         <v>0</v>
       </c>
       <c r="R50" s="1">
@@ -13072,7 +13030,7 @@
       <c r="M51">
         <v>0</v>
       </c>
-      <c r="O51">
+      <c r="O51" s="1">
         <v>0</v>
       </c>
       <c r="R51" s="1">
@@ -13115,7 +13073,7 @@
       <c r="M52">
         <v>0</v>
       </c>
-      <c r="O52">
+      <c r="O52" s="1">
         <v>0</v>
       </c>
       <c r="R52" s="1">
@@ -13158,7 +13116,7 @@
       <c r="M53">
         <v>0</v>
       </c>
-      <c r="O53">
+      <c r="O53" s="1">
         <v>0</v>
       </c>
       <c r="R53" s="1">
@@ -13201,7 +13159,7 @@
       <c r="M54">
         <v>0</v>
       </c>
-      <c r="O54">
+      <c r="O54" s="1">
         <v>0</v>
       </c>
       <c r="R54" s="1">
@@ -13244,7 +13202,7 @@
       <c r="M55">
         <v>0</v>
       </c>
-      <c r="O55">
+      <c r="O55" s="1">
         <v>0</v>
       </c>
       <c r="R55" s="1">
@@ -13287,7 +13245,7 @@
       <c r="M56">
         <v>0</v>
       </c>
-      <c r="O56">
+      <c r="O56" s="1">
         <v>0</v>
       </c>
       <c r="R56" s="1">
@@ -13330,7 +13288,7 @@
       <c r="M57">
         <v>0</v>
       </c>
-      <c r="O57">
+      <c r="O57" s="1">
         <v>0</v>
       </c>
       <c r="R57" s="1">
@@ -13373,7 +13331,7 @@
       <c r="M58">
         <v>0</v>
       </c>
-      <c r="O58">
+      <c r="O58" s="1">
         <v>0</v>
       </c>
       <c r="R58" s="1">
@@ -13416,7 +13374,7 @@
       <c r="M59">
         <v>0</v>
       </c>
-      <c r="O59">
+      <c r="O59" s="1">
         <v>0</v>
       </c>
       <c r="R59" s="1">
@@ -13459,7 +13417,7 @@
       <c r="M60">
         <v>0</v>
       </c>
-      <c r="O60">
+      <c r="O60" s="1">
         <v>0</v>
       </c>
       <c r="R60" s="1">
@@ -13502,7 +13460,7 @@
       <c r="M61">
         <v>0</v>
       </c>
-      <c r="O61">
+      <c r="O61" s="1">
         <v>0</v>
       </c>
       <c r="R61" s="1">
@@ -13545,7 +13503,7 @@
       <c r="M62">
         <v>0</v>
       </c>
-      <c r="O62">
+      <c r="O62" s="1">
         <v>0</v>
       </c>
       <c r="R62" s="1">
@@ -13588,7 +13546,7 @@
       <c r="M63">
         <v>0</v>
       </c>
-      <c r="O63">
+      <c r="O63" s="1">
         <v>0</v>
       </c>
       <c r="R63" s="1">
@@ -13631,7 +13589,7 @@
       <c r="M64">
         <v>0</v>
       </c>
-      <c r="O64">
+      <c r="O64" s="1">
         <v>0</v>
       </c>
       <c r="R64" s="1">
@@ -13674,7 +13632,7 @@
       <c r="M65">
         <v>0</v>
       </c>
-      <c r="O65">
+      <c r="O65" s="1">
         <v>0</v>
       </c>
       <c r="R65" s="1">
@@ -13717,7 +13675,7 @@
       <c r="M66">
         <v>0</v>
       </c>
-      <c r="O66">
+      <c r="O66" s="1">
         <v>0</v>
       </c>
       <c r="R66" s="1">
@@ -13760,7 +13718,7 @@
       <c r="M67">
         <v>0</v>
       </c>
-      <c r="O67">
+      <c r="O67" s="1">
         <v>0</v>
       </c>
       <c r="R67" s="1">
@@ -13803,7 +13761,7 @@
       <c r="M68">
         <v>0</v>
       </c>
-      <c r="O68">
+      <c r="O68" s="1">
         <v>0</v>
       </c>
       <c r="R68" s="1">
@@ -13847,7 +13805,7 @@
       <c r="M69">
         <v>0</v>
       </c>
-      <c r="O69">
+      <c r="O69" s="1">
         <v>0</v>
       </c>
       <c r="R69" s="1">
@@ -13891,7 +13849,7 @@
       <c r="M70">
         <v>0</v>
       </c>
-      <c r="O70">
+      <c r="O70" s="1">
         <v>0</v>
       </c>
       <c r="R70" s="1">
@@ -13931,7 +13889,7 @@
       <c r="M71">
         <v>0</v>
       </c>
-      <c r="O71">
+      <c r="O71" s="1">
         <v>0</v>
       </c>
       <c r="R71" s="1">
@@ -13967,7 +13925,7 @@
       <c r="M72">
         <v>0</v>
       </c>
-      <c r="O72">
+      <c r="O72" s="1">
         <v>0</v>
       </c>
       <c r="R72" s="1">
@@ -15304,9 +15262,6 @@
     <row r="10" hidden="1" ht="15" customHeight="1"/>
     <row r="11" ht="23.25" customHeight="1"/>
     <row r="12" ht="23.25" customHeight="1">
-      <c r="D12">
-        <v>0</v>
-      </c>
       <c r="G12" s="1">
         <f>H2</f>
         <v>30641.975</v>
@@ -15319,18 +15274,7 @@
         <v>0</v>
       </c>
       <c r="J12">
-        <v>0</v>
-      </c>
-      <c r="K12">
-        <v>0</v>
-      </c>
-      <c r="L12">
-        <v>0</v>
-      </c>
-      <c r="M12">
-        <v>0</v>
-      </c>
-      <c r="O12">
+        <f>(K12+M12+L12)</f>
         <v>0</v>
       </c>
     </row>
@@ -15375,7 +15319,7 @@
       <c r="M13">
         <v>0</v>
       </c>
-      <c r="O13">
+      <c r="O13" s="1">
         <v>0</v>
       </c>
     </row>
@@ -15415,7 +15359,7 @@
       <c r="M14">
         <v>0</v>
       </c>
-      <c r="O14">
+      <c r="O14" s="1">
         <v>0</v>
       </c>
       <c r="R14" s="1">
@@ -15459,7 +15403,7 @@
       <c r="M15">
         <v>0</v>
       </c>
-      <c r="O15">
+      <c r="O15" s="1">
         <v>0</v>
       </c>
       <c r="R15" s="1">
@@ -15506,7 +15450,7 @@
       <c r="M16">
         <v>0</v>
       </c>
-      <c r="O16">
+      <c r="O16" s="1">
         <v>0</v>
       </c>
       <c r="R16" s="1">
@@ -15550,7 +15494,7 @@
       <c r="M17">
         <v>0</v>
       </c>
-      <c r="O17">
+      <c r="O17" s="1">
         <v>0</v>
       </c>
       <c r="R17" s="1">
@@ -15594,7 +15538,7 @@
       <c r="M18">
         <v>0</v>
       </c>
-      <c r="O18">
+      <c r="O18" s="1">
         <v>0</v>
       </c>
       <c r="R18" s="1">
@@ -15641,7 +15585,7 @@
       <c r="M19">
         <v>0</v>
       </c>
-      <c r="O19">
+      <c r="O19" s="1">
         <v>0</v>
       </c>
       <c r="R19" s="1">
@@ -15684,7 +15628,7 @@
       <c r="M20">
         <v>0</v>
       </c>
-      <c r="O20">
+      <c r="O20" s="1">
         <v>0</v>
       </c>
       <c r="R20" s="1">
@@ -15728,7 +15672,7 @@
       <c r="M21">
         <v>0</v>
       </c>
-      <c r="O21">
+      <c r="O21" s="1">
         <v>0</v>
       </c>
       <c r="R21" s="1">
@@ -15771,7 +15715,7 @@
       <c r="M22">
         <v>0</v>
       </c>
-      <c r="O22">
+      <c r="O22" s="1">
         <v>0</v>
       </c>
       <c r="R22" s="1">
@@ -15818,7 +15762,7 @@
       <c r="M23">
         <v>0</v>
       </c>
-      <c r="O23">
+      <c r="O23" s="1">
         <v>0</v>
       </c>
       <c r="R23" s="1">
@@ -15862,7 +15806,7 @@
       <c r="M24">
         <v>0</v>
       </c>
-      <c r="O24">
+      <c r="O24" s="1">
         <v>0</v>
       </c>
       <c r="R24" s="1">
@@ -15906,7 +15850,7 @@
       <c r="M25">
         <v>0</v>
       </c>
-      <c r="O25">
+      <c r="O25" s="1">
         <v>0</v>
       </c>
       <c r="R25" s="1">
@@ -15953,7 +15897,7 @@
       <c r="M26">
         <v>0</v>
       </c>
-      <c r="O26">
+      <c r="O26" s="1">
         <v>0</v>
       </c>
       <c r="R26" s="1">
@@ -15997,7 +15941,7 @@
       <c r="M27">
         <v>0</v>
       </c>
-      <c r="O27">
+      <c r="O27" s="1">
         <v>0</v>
       </c>
       <c r="R27" s="1">
@@ -16041,7 +15985,7 @@
       <c r="M28">
         <v>0</v>
       </c>
-      <c r="O28">
+      <c r="O28" s="1">
         <v>0</v>
       </c>
       <c r="R28" s="1">
@@ -16085,7 +16029,7 @@
       <c r="M29">
         <v>0</v>
       </c>
-      <c r="O29">
+      <c r="O29" s="1">
         <v>0</v>
       </c>
       <c r="R29" s="1">
@@ -16132,7 +16076,7 @@
       <c r="M30">
         <v>0</v>
       </c>
-      <c r="O30">
+      <c r="O30" s="1">
         <v>0</v>
       </c>
       <c r="R30" s="1">
@@ -16176,7 +16120,7 @@
       <c r="M31">
         <v>0</v>
       </c>
-      <c r="O31">
+      <c r="O31" s="1">
         <v>0</v>
       </c>
       <c r="R31" s="1">
@@ -16220,7 +16164,7 @@
       <c r="M32">
         <v>0</v>
       </c>
-      <c r="O32">
+      <c r="O32" s="1">
         <v>0</v>
       </c>
       <c r="R32" s="1">
@@ -16267,7 +16211,7 @@
       <c r="M33">
         <v>0</v>
       </c>
-      <c r="O33">
+      <c r="O33" s="1">
         <v>0</v>
       </c>
       <c r="R33" s="1">
@@ -16311,7 +16255,7 @@
       <c r="M34">
         <v>0</v>
       </c>
-      <c r="O34">
+      <c r="O34" s="1">
         <v>0</v>
       </c>
       <c r="R34" s="1">
@@ -16355,7 +16299,7 @@
       <c r="M35">
         <v>0</v>
       </c>
-      <c r="O35">
+      <c r="O35" s="1">
         <v>0</v>
       </c>
       <c r="R35" s="1">
@@ -16399,7 +16343,7 @@
       <c r="M36">
         <v>0</v>
       </c>
-      <c r="O36">
+      <c r="O36" s="1">
         <v>0</v>
       </c>
       <c r="R36" s="1">
@@ -16443,7 +16387,7 @@
       <c r="M37">
         <v>0</v>
       </c>
-      <c r="O37">
+      <c r="O37" s="1">
         <v>0</v>
       </c>
       <c r="R37" s="1">
@@ -16487,7 +16431,7 @@
       <c r="M38">
         <v>0</v>
       </c>
-      <c r="O38">
+      <c r="O38" s="1">
         <v>0</v>
       </c>
       <c r="R38" s="1">
@@ -16531,7 +16475,7 @@
       <c r="M39">
         <v>0</v>
       </c>
-      <c r="O39">
+      <c r="O39" s="1">
         <v>0</v>
       </c>
       <c r="R39" s="1">
@@ -16575,7 +16519,7 @@
       <c r="M40">
         <v>0</v>
       </c>
-      <c r="O40">
+      <c r="O40" s="1">
         <v>0</v>
       </c>
       <c r="R40" s="1">
@@ -16619,7 +16563,7 @@
       <c r="M41">
         <v>0</v>
       </c>
-      <c r="O41">
+      <c r="O41" s="1">
         <v>0</v>
       </c>
       <c r="R41" s="1">
@@ -16663,7 +16607,7 @@
       <c r="M42">
         <v>0</v>
       </c>
-      <c r="O42">
+      <c r="O42" s="1">
         <v>0</v>
       </c>
       <c r="R42" s="1">
@@ -16707,7 +16651,7 @@
       <c r="M43">
         <v>0</v>
       </c>
-      <c r="O43">
+      <c r="O43" s="1">
         <v>0</v>
       </c>
       <c r="R43" s="1">
@@ -16751,7 +16695,7 @@
       <c r="M44">
         <v>0</v>
       </c>
-      <c r="O44">
+      <c r="O44" s="1">
         <v>0</v>
       </c>
       <c r="R44" s="1">
@@ -16794,7 +16738,7 @@
       <c r="M45">
         <v>0</v>
       </c>
-      <c r="O45">
+      <c r="O45" s="1">
         <v>0</v>
       </c>
       <c r="R45" s="1">
@@ -16837,7 +16781,7 @@
       <c r="M46">
         <v>0</v>
       </c>
-      <c r="O46">
+      <c r="O46" s="1">
         <v>0</v>
       </c>
       <c r="R46" s="1">
@@ -16880,7 +16824,7 @@
       <c r="M47">
         <v>0</v>
       </c>
-      <c r="O47">
+      <c r="O47" s="1">
         <v>0</v>
       </c>
       <c r="R47" s="1">
@@ -16923,7 +16867,7 @@
       <c r="M48">
         <v>0</v>
       </c>
-      <c r="O48">
+      <c r="O48" s="1">
         <v>0</v>
       </c>
       <c r="R48" s="1">
@@ -16966,7 +16910,7 @@
       <c r="M49">
         <v>0</v>
       </c>
-      <c r="O49">
+      <c r="O49" s="1">
         <v>0</v>
       </c>
       <c r="R49" s="1">
@@ -17009,7 +16953,7 @@
       <c r="M50">
         <v>0</v>
       </c>
-      <c r="O50">
+      <c r="O50" s="1">
         <v>0</v>
       </c>
       <c r="R50" s="1">
@@ -17052,7 +16996,7 @@
       <c r="M51">
         <v>0</v>
       </c>
-      <c r="O51">
+      <c r="O51" s="1">
         <v>0</v>
       </c>
       <c r="R51" s="1">
@@ -17095,7 +17039,7 @@
       <c r="M52">
         <v>0</v>
       </c>
-      <c r="O52">
+      <c r="O52" s="1">
         <v>0</v>
       </c>
       <c r="R52" s="1">
@@ -17138,7 +17082,7 @@
       <c r="M53">
         <v>0</v>
       </c>
-      <c r="O53">
+      <c r="O53" s="1">
         <v>0</v>
       </c>
       <c r="R53" s="1">
@@ -17181,7 +17125,7 @@
       <c r="M54">
         <v>0</v>
       </c>
-      <c r="O54">
+      <c r="O54" s="1">
         <v>0</v>
       </c>
       <c r="R54" s="1">
@@ -17224,7 +17168,7 @@
       <c r="M55">
         <v>0</v>
       </c>
-      <c r="O55">
+      <c r="O55" s="1">
         <v>0</v>
       </c>
       <c r="R55" s="1">
@@ -17267,7 +17211,7 @@
       <c r="M56">
         <v>0</v>
       </c>
-      <c r="O56">
+      <c r="O56" s="1">
         <v>0</v>
       </c>
       <c r="R56" s="1">
@@ -17310,7 +17254,7 @@
       <c r="M57">
         <v>0</v>
       </c>
-      <c r="O57">
+      <c r="O57" s="1">
         <v>0</v>
       </c>
       <c r="R57" s="1">
@@ -17353,7 +17297,7 @@
       <c r="M58">
         <v>0</v>
       </c>
-      <c r="O58">
+      <c r="O58" s="1">
         <v>0</v>
       </c>
       <c r="R58" s="1">
@@ -17396,7 +17340,7 @@
       <c r="M59">
         <v>0</v>
       </c>
-      <c r="O59">
+      <c r="O59" s="1">
         <v>0</v>
       </c>
       <c r="R59" s="1">
@@ -17439,7 +17383,7 @@
       <c r="M60">
         <v>0</v>
       </c>
-      <c r="O60">
+      <c r="O60" s="1">
         <v>0</v>
       </c>
       <c r="R60" s="1">
@@ -17482,7 +17426,7 @@
       <c r="M61">
         <v>0</v>
       </c>
-      <c r="O61">
+      <c r="O61" s="1">
         <v>0</v>
       </c>
       <c r="R61" s="1">
@@ -17525,7 +17469,7 @@
       <c r="M62">
         <v>0</v>
       </c>
-      <c r="O62">
+      <c r="O62" s="1">
         <v>0</v>
       </c>
       <c r="R62" s="1">
@@ -17568,7 +17512,7 @@
       <c r="M63">
         <v>0</v>
       </c>
-      <c r="O63">
+      <c r="O63" s="1">
         <v>0</v>
       </c>
       <c r="R63" s="1">
@@ -17611,7 +17555,7 @@
       <c r="M64">
         <v>0</v>
       </c>
-      <c r="O64">
+      <c r="O64" s="1">
         <v>0</v>
       </c>
       <c r="R64" s="1">
@@ -17654,7 +17598,7 @@
       <c r="M65">
         <v>0</v>
       </c>
-      <c r="O65">
+      <c r="O65" s="1">
         <v>0</v>
       </c>
       <c r="R65" s="1">
@@ -17697,7 +17641,7 @@
       <c r="M66">
         <v>0</v>
       </c>
-      <c r="O66">
+      <c r="O66" s="1">
         <v>0</v>
       </c>
       <c r="R66" s="1">
@@ -17740,7 +17684,7 @@
       <c r="M67">
         <v>0</v>
       </c>
-      <c r="O67">
+      <c r="O67" s="1">
         <v>0</v>
       </c>
       <c r="R67" s="1">
@@ -17783,7 +17727,7 @@
       <c r="M68">
         <v>0</v>
       </c>
-      <c r="O68">
+      <c r="O68" s="1">
         <v>0</v>
       </c>
       <c r="R68" s="1">
@@ -17827,7 +17771,7 @@
       <c r="M69">
         <v>0</v>
       </c>
-      <c r="O69">
+      <c r="O69" s="1">
         <v>0</v>
       </c>
       <c r="R69" s="1">
@@ -17871,7 +17815,7 @@
       <c r="M70">
         <v>0</v>
       </c>
-      <c r="O70">
+      <c r="O70" s="1">
         <v>0</v>
       </c>
       <c r="R70" s="1">
@@ -17911,7 +17855,7 @@
       <c r="M71">
         <v>0</v>
       </c>
-      <c r="O71">
+      <c r="O71" s="1">
         <v>0</v>
       </c>
       <c r="R71" s="1">
@@ -17947,7 +17891,7 @@
       <c r="M72">
         <v>0</v>
       </c>
-      <c r="O72">
+      <c r="O72" s="1">
         <v>0</v>
       </c>
       <c r="R72" s="1">
@@ -19283,9 +19227,6 @@
     <row r="10" hidden="1" ht="15" customHeight="1"/>
     <row r="11" ht="23.25" customHeight="1"/>
     <row r="12" ht="23.25" customHeight="1">
-      <c r="D12">
-        <v>0</v>
-      </c>
       <c r="G12" s="1">
         <f>H2</f>
         <v>14984.125</v>
@@ -19298,18 +19239,7 @@
         <v>0</v>
       </c>
       <c r="J12">
-        <v>0</v>
-      </c>
-      <c r="K12">
-        <v>0</v>
-      </c>
-      <c r="L12">
-        <v>0</v>
-      </c>
-      <c r="M12">
-        <v>0</v>
-      </c>
-      <c r="O12">
+        <f>(K12+M12+L12)</f>
         <v>0</v>
       </c>
     </row>
@@ -19354,7 +19284,7 @@
       <c r="M13">
         <v>0</v>
       </c>
-      <c r="O13">
+      <c r="O13" s="1">
         <v>0</v>
       </c>
     </row>
@@ -19397,7 +19327,7 @@
       <c r="M14">
         <v>0</v>
       </c>
-      <c r="O14">
+      <c r="O14" s="1">
         <v>0</v>
       </c>
       <c r="R14" s="1">
@@ -19441,7 +19371,7 @@
       <c r="M15">
         <v>0</v>
       </c>
-      <c r="O15">
+      <c r="O15" s="1">
         <v>0</v>
       </c>
       <c r="R15" s="1">
@@ -19485,7 +19415,7 @@
       <c r="M16">
         <v>0</v>
       </c>
-      <c r="O16">
+      <c r="O16" s="1">
         <v>0</v>
       </c>
       <c r="R16" s="1">
@@ -19529,7 +19459,7 @@
       <c r="M17">
         <v>0</v>
       </c>
-      <c r="O17">
+      <c r="O17" s="1">
         <v>0</v>
       </c>
       <c r="R17" s="1">
@@ -19576,7 +19506,7 @@
       <c r="M18">
         <v>0</v>
       </c>
-      <c r="O18">
+      <c r="O18" s="1">
         <v>0</v>
       </c>
       <c r="R18" s="1">
@@ -19620,7 +19550,7 @@
       <c r="M19">
         <v>0</v>
       </c>
-      <c r="O19">
+      <c r="O19" s="1">
         <v>0</v>
       </c>
       <c r="R19" s="1">
@@ -19663,7 +19593,7 @@
       <c r="M20">
         <v>0</v>
       </c>
-      <c r="O20">
+      <c r="O20" s="1">
         <v>0</v>
       </c>
       <c r="R20" s="1">
@@ -19707,7 +19637,7 @@
       <c r="M21">
         <v>0</v>
       </c>
-      <c r="O21">
+      <c r="O21" s="1">
         <v>0</v>
       </c>
       <c r="R21" s="1">
@@ -19753,7 +19683,7 @@
       <c r="M22">
         <v>0</v>
       </c>
-      <c r="O22">
+      <c r="O22" s="1">
         <v>0</v>
       </c>
       <c r="R22" s="1">
@@ -19797,7 +19727,7 @@
       <c r="M23">
         <v>0</v>
       </c>
-      <c r="O23">
+      <c r="O23" s="1">
         <v>0</v>
       </c>
       <c r="R23" s="1">
@@ -19841,7 +19771,7 @@
       <c r="M24">
         <v>0</v>
       </c>
-      <c r="O24">
+      <c r="O24" s="1">
         <v>0</v>
       </c>
       <c r="R24" s="1">
@@ -19888,7 +19818,7 @@
       <c r="M25">
         <v>0</v>
       </c>
-      <c r="O25">
+      <c r="O25" s="1">
         <v>0</v>
       </c>
       <c r="R25" s="1">
@@ -19932,7 +19862,7 @@
       <c r="M26">
         <v>0</v>
       </c>
-      <c r="O26">
+      <c r="O26" s="1">
         <v>0</v>
       </c>
       <c r="R26" s="1">
@@ -19976,7 +19906,7 @@
       <c r="M27">
         <v>0</v>
       </c>
-      <c r="O27">
+      <c r="O27" s="1">
         <v>0</v>
       </c>
       <c r="R27" s="1">
@@ -20020,7 +19950,7 @@
       <c r="M28">
         <v>0</v>
       </c>
-      <c r="O28">
+      <c r="O28" s="1">
         <v>0</v>
       </c>
       <c r="R28" s="1">
@@ -20067,7 +19997,7 @@
       <c r="M29">
         <v>0</v>
       </c>
-      <c r="O29">
+      <c r="O29" s="1">
         <v>0</v>
       </c>
       <c r="R29" s="1">
@@ -20111,7 +20041,7 @@
       <c r="M30">
         <v>0</v>
       </c>
-      <c r="O30">
+      <c r="O30" s="1">
         <v>0</v>
       </c>
       <c r="R30" s="1">
@@ -20155,7 +20085,7 @@
       <c r="M31">
         <v>0</v>
       </c>
-      <c r="O31">
+      <c r="O31" s="1">
         <v>0</v>
       </c>
       <c r="R31" s="1">
@@ -20202,7 +20132,7 @@
       <c r="M32">
         <v>0</v>
       </c>
-      <c r="O32">
+      <c r="O32" s="1">
         <v>0</v>
       </c>
       <c r="R32" s="1">
@@ -20246,7 +20176,7 @@
       <c r="M33">
         <v>0</v>
       </c>
-      <c r="O33">
+      <c r="O33" s="1">
         <v>0</v>
       </c>
       <c r="R33" s="1">
@@ -20290,7 +20220,7 @@
       <c r="M34">
         <v>0</v>
       </c>
-      <c r="O34">
+      <c r="O34" s="1">
         <v>0</v>
       </c>
       <c r="R34" s="1">
@@ -20334,7 +20264,7 @@
       <c r="M35">
         <v>0</v>
       </c>
-      <c r="O35">
+      <c r="O35" s="1">
         <v>0</v>
       </c>
       <c r="R35" s="1">
@@ -20378,7 +20308,7 @@
       <c r="M36">
         <v>0</v>
       </c>
-      <c r="O36">
+      <c r="O36" s="1">
         <v>0</v>
       </c>
       <c r="R36" s="1">
@@ -20422,7 +20352,7 @@
       <c r="M37">
         <v>0</v>
       </c>
-      <c r="O37">
+      <c r="O37" s="1">
         <v>0</v>
       </c>
       <c r="R37" s="1">
@@ -20466,7 +20396,7 @@
       <c r="M38">
         <v>0</v>
       </c>
-      <c r="O38">
+      <c r="O38" s="1">
         <v>0</v>
       </c>
       <c r="R38" s="1">
@@ -20510,7 +20440,7 @@
       <c r="M39">
         <v>0</v>
       </c>
-      <c r="O39">
+      <c r="O39" s="1">
         <v>0</v>
       </c>
       <c r="R39" s="1">
@@ -20554,7 +20484,7 @@
       <c r="M40">
         <v>0</v>
       </c>
-      <c r="O40">
+      <c r="O40" s="1">
         <v>0</v>
       </c>
       <c r="R40" s="1">
@@ -20598,7 +20528,7 @@
       <c r="M41">
         <v>0</v>
       </c>
-      <c r="O41">
+      <c r="O41" s="1">
         <v>0</v>
       </c>
       <c r="R41" s="1">
@@ -20642,7 +20572,7 @@
       <c r="M42">
         <v>0</v>
       </c>
-      <c r="O42">
+      <c r="O42" s="1">
         <v>0</v>
       </c>
       <c r="R42" s="1">
@@ -20686,7 +20616,7 @@
       <c r="M43">
         <v>0</v>
       </c>
-      <c r="O43">
+      <c r="O43" s="1">
         <v>0</v>
       </c>
       <c r="R43" s="1">
@@ -20730,7 +20660,7 @@
       <c r="M44">
         <v>0</v>
       </c>
-      <c r="O44">
+      <c r="O44" s="1">
         <v>0</v>
       </c>
       <c r="R44" s="1">
@@ -20773,7 +20703,7 @@
       <c r="M45">
         <v>0</v>
       </c>
-      <c r="O45">
+      <c r="O45" s="1">
         <v>0</v>
       </c>
       <c r="R45" s="1">
@@ -20816,7 +20746,7 @@
       <c r="M46">
         <v>0</v>
       </c>
-      <c r="O46">
+      <c r="O46" s="1">
         <v>0</v>
       </c>
       <c r="R46" s="1">
@@ -20859,7 +20789,7 @@
       <c r="M47">
         <v>0</v>
       </c>
-      <c r="O47">
+      <c r="O47" s="1">
         <v>0</v>
       </c>
       <c r="R47" s="1">
@@ -20902,7 +20832,7 @@
       <c r="M48">
         <v>0</v>
       </c>
-      <c r="O48">
+      <c r="O48" s="1">
         <v>0</v>
       </c>
       <c r="R48" s="1">
@@ -20945,7 +20875,7 @@
       <c r="M49">
         <v>0</v>
       </c>
-      <c r="O49">
+      <c r="O49" s="1">
         <v>0</v>
       </c>
       <c r="R49" s="1">
@@ -20988,7 +20918,7 @@
       <c r="M50">
         <v>0</v>
       </c>
-      <c r="O50">
+      <c r="O50" s="1">
         <v>0</v>
       </c>
       <c r="R50" s="1">
@@ -21031,7 +20961,7 @@
       <c r="M51">
         <v>0</v>
       </c>
-      <c r="O51">
+      <c r="O51" s="1">
         <v>0</v>
       </c>
       <c r="R51" s="1">
@@ -21074,7 +21004,7 @@
       <c r="M52">
         <v>0</v>
       </c>
-      <c r="O52">
+      <c r="O52" s="1">
         <v>0</v>
       </c>
       <c r="R52" s="1">
@@ -21117,7 +21047,7 @@
       <c r="M53">
         <v>0</v>
       </c>
-      <c r="O53">
+      <c r="O53" s="1">
         <v>0</v>
       </c>
       <c r="R53" s="1">
@@ -21160,7 +21090,7 @@
       <c r="M54">
         <v>0</v>
       </c>
-      <c r="O54">
+      <c r="O54" s="1">
         <v>0</v>
       </c>
       <c r="R54" s="1">
@@ -21203,7 +21133,7 @@
       <c r="M55">
         <v>0</v>
       </c>
-      <c r="O55">
+      <c r="O55" s="1">
         <v>0</v>
       </c>
       <c r="R55" s="1">
@@ -21246,7 +21176,7 @@
       <c r="M56">
         <v>0</v>
       </c>
-      <c r="O56">
+      <c r="O56" s="1">
         <v>0</v>
       </c>
       <c r="R56" s="1">
@@ -21289,7 +21219,7 @@
       <c r="M57">
         <v>0</v>
       </c>
-      <c r="O57">
+      <c r="O57" s="1">
         <v>0</v>
       </c>
       <c r="R57" s="1">
@@ -21332,7 +21262,7 @@
       <c r="M58">
         <v>0</v>
       </c>
-      <c r="O58">
+      <c r="O58" s="1">
         <v>0</v>
       </c>
       <c r="R58" s="1">
@@ -21375,7 +21305,7 @@
       <c r="M59">
         <v>0</v>
       </c>
-      <c r="O59">
+      <c r="O59" s="1">
         <v>0</v>
       </c>
       <c r="R59" s="1">
@@ -21418,7 +21348,7 @@
       <c r="M60">
         <v>0</v>
       </c>
-      <c r="O60">
+      <c r="O60" s="1">
         <v>0</v>
       </c>
       <c r="R60" s="1">
@@ -21461,7 +21391,7 @@
       <c r="M61">
         <v>0</v>
       </c>
-      <c r="O61">
+      <c r="O61" s="1">
         <v>0</v>
       </c>
       <c r="R61" s="1">
@@ -21504,7 +21434,7 @@
       <c r="M62">
         <v>0</v>
       </c>
-      <c r="O62">
+      <c r="O62" s="1">
         <v>0</v>
       </c>
       <c r="R62" s="1">
@@ -21547,7 +21477,7 @@
       <c r="M63">
         <v>0</v>
       </c>
-      <c r="O63">
+      <c r="O63" s="1">
         <v>0</v>
       </c>
       <c r="R63" s="1">
@@ -21590,7 +21520,7 @@
       <c r="M64">
         <v>0</v>
       </c>
-      <c r="O64">
+      <c r="O64" s="1">
         <v>0</v>
       </c>
       <c r="R64" s="1">
@@ -21633,7 +21563,7 @@
       <c r="M65">
         <v>0</v>
       </c>
-      <c r="O65">
+      <c r="O65" s="1">
         <v>0</v>
       </c>
       <c r="R65" s="1">
@@ -21676,7 +21606,7 @@
       <c r="M66">
         <v>0</v>
       </c>
-      <c r="O66">
+      <c r="O66" s="1">
         <v>0</v>
       </c>
       <c r="R66" s="1">
@@ -21719,7 +21649,7 @@
       <c r="M67">
         <v>0</v>
       </c>
-      <c r="O67">
+      <c r="O67" s="1">
         <v>0</v>
       </c>
       <c r="R67" s="1">
@@ -21762,7 +21692,7 @@
       <c r="M68">
         <v>0</v>
       </c>
-      <c r="O68">
+      <c r="O68" s="1">
         <v>0</v>
       </c>
       <c r="R68" s="1">
@@ -21806,7 +21736,7 @@
       <c r="M69">
         <v>0</v>
       </c>
-      <c r="O69">
+      <c r="O69" s="1">
         <v>0</v>
       </c>
       <c r="R69" s="1">
@@ -21850,7 +21780,7 @@
       <c r="M70">
         <v>0</v>
       </c>
-      <c r="O70">
+      <c r="O70" s="1">
         <v>0</v>
       </c>
       <c r="R70" s="1">
@@ -21890,7 +21820,7 @@
       <c r="M71">
         <v>0</v>
       </c>
-      <c r="O71">
+      <c r="O71" s="1">
         <v>0</v>
       </c>
       <c r="R71" s="1">
@@ -21926,7 +21856,7 @@
       <c r="M72">
         <v>0</v>
       </c>
-      <c r="O72">
+      <c r="O72" s="1">
         <v>0</v>
       </c>
       <c r="R72" s="1">
@@ -23263,9 +23193,6 @@
     <row r="10" hidden="1" ht="15" customHeight="1"/>
     <row r="11" ht="23.25" customHeight="1"/>
     <row r="12" ht="23.25" customHeight="1">
-      <c r="D12">
-        <v>0</v>
-      </c>
       <c r="G12" s="1">
         <f>H2</f>
         <v>32175</v>
@@ -23278,18 +23205,7 @@
         <v>0</v>
       </c>
       <c r="J12">
-        <v>0</v>
-      </c>
-      <c r="K12">
-        <v>0</v>
-      </c>
-      <c r="L12">
-        <v>0</v>
-      </c>
-      <c r="M12">
-        <v>0</v>
-      </c>
-      <c r="O12">
+        <f>(K12+M12+L12)</f>
         <v>0</v>
       </c>
     </row>
@@ -23334,7 +23250,7 @@
       <c r="M13">
         <v>0</v>
       </c>
-      <c r="O13">
+      <c r="O13" s="1">
         <v>0</v>
       </c>
     </row>
@@ -23377,7 +23293,7 @@
       <c r="M14">
         <v>0</v>
       </c>
-      <c r="O14">
+      <c r="O14" s="1">
         <v>0</v>
       </c>
       <c r="R14" s="1">
@@ -23421,7 +23337,7 @@
       <c r="M15">
         <v>0</v>
       </c>
-      <c r="O15">
+      <c r="O15" s="1">
         <v>0</v>
       </c>
       <c r="R15" s="1">
@@ -23468,7 +23384,7 @@
       <c r="M16">
         <v>0</v>
       </c>
-      <c r="O16">
+      <c r="O16" s="1">
         <v>0</v>
       </c>
       <c r="R16" s="1">
@@ -23512,7 +23428,7 @@
       <c r="M17">
         <v>0</v>
       </c>
-      <c r="O17">
+      <c r="O17" s="1">
         <v>0</v>
       </c>
       <c r="R17" s="1">
@@ -23556,7 +23472,7 @@
       <c r="M18">
         <v>0</v>
       </c>
-      <c r="O18">
+      <c r="O18" s="1">
         <v>0</v>
       </c>
       <c r="R18" s="1">
@@ -23600,7 +23516,7 @@
       <c r="M19">
         <v>0</v>
       </c>
-      <c r="O19">
+      <c r="O19" s="1">
         <v>0</v>
       </c>
       <c r="R19" s="1">
@@ -23646,7 +23562,7 @@
       <c r="M20">
         <v>0</v>
       </c>
-      <c r="O20">
+      <c r="O20" s="1">
         <v>0</v>
       </c>
       <c r="R20" s="1">
@@ -23690,7 +23606,7 @@
       <c r="M21">
         <v>0</v>
       </c>
-      <c r="O21">
+      <c r="O21" s="1">
         <v>0</v>
       </c>
       <c r="R21" s="1">
@@ -23733,7 +23649,7 @@
       <c r="M22">
         <v>0</v>
       </c>
-      <c r="O22">
+      <c r="O22" s="1">
         <v>0</v>
       </c>
       <c r="R22" s="1">
@@ -23780,7 +23696,7 @@
       <c r="M23">
         <v>0</v>
       </c>
-      <c r="O23">
+      <c r="O23" s="1">
         <v>0</v>
       </c>
       <c r="R23" s="1">
@@ -23824,7 +23740,7 @@
       <c r="M24">
         <v>0</v>
       </c>
-      <c r="O24">
+      <c r="O24" s="1">
         <v>0</v>
       </c>
       <c r="R24" s="1">
@@ -23868,7 +23784,7 @@
       <c r="M25">
         <v>0</v>
       </c>
-      <c r="O25">
+      <c r="O25" s="1">
         <v>0</v>
       </c>
       <c r="R25" s="1">
@@ -23912,7 +23828,7 @@
       <c r="M26">
         <v>0</v>
       </c>
-      <c r="O26">
+      <c r="O26" s="1">
         <v>0</v>
       </c>
       <c r="R26" s="1">
@@ -23958,7 +23874,7 @@
       <c r="M27">
         <v>0</v>
       </c>
-      <c r="O27">
+      <c r="O27" s="1">
         <v>0</v>
       </c>
       <c r="R27" s="1">
@@ -24002,7 +23918,7 @@
       <c r="M28">
         <v>0</v>
       </c>
-      <c r="O28">
+      <c r="O28" s="1">
         <v>0</v>
       </c>
       <c r="R28" s="1">
@@ -24046,7 +23962,7 @@
       <c r="M29">
         <v>0</v>
       </c>
-      <c r="O29">
+      <c r="O29" s="1">
         <v>0</v>
       </c>
       <c r="R29" s="1">
@@ -24093,7 +24009,7 @@
       <c r="M30">
         <v>0</v>
       </c>
-      <c r="O30">
+      <c r="O30" s="1">
         <v>0</v>
       </c>
       <c r="R30" s="1">
@@ -24137,7 +24053,7 @@
       <c r="M31">
         <v>0</v>
       </c>
-      <c r="O31">
+      <c r="O31" s="1">
         <v>0</v>
       </c>
       <c r="R31" s="1">
@@ -24181,7 +24097,7 @@
       <c r="M32">
         <v>0</v>
       </c>
-      <c r="O32">
+      <c r="O32" s="1">
         <v>0</v>
       </c>
       <c r="R32" s="1">
@@ -24225,7 +24141,7 @@
       <c r="M33">
         <v>0</v>
       </c>
-      <c r="O33">
+      <c r="O33" s="1">
         <v>0</v>
       </c>
       <c r="R33" s="1">
@@ -24269,7 +24185,7 @@
       <c r="M34">
         <v>0</v>
       </c>
-      <c r="O34">
+      <c r="O34" s="1">
         <v>0</v>
       </c>
       <c r="R34" s="1">
@@ -24313,7 +24229,7 @@
       <c r="M35">
         <v>0</v>
       </c>
-      <c r="O35">
+      <c r="O35" s="1">
         <v>0</v>
       </c>
       <c r="R35" s="1">
@@ -24357,7 +24273,7 @@
       <c r="M36">
         <v>0</v>
       </c>
-      <c r="O36">
+      <c r="O36" s="1">
         <v>0</v>
       </c>
       <c r="R36" s="1">
@@ -24401,7 +24317,7 @@
       <c r="M37">
         <v>0</v>
       </c>
-      <c r="O37">
+      <c r="O37" s="1">
         <v>0</v>
       </c>
       <c r="R37" s="1">
@@ -24445,7 +24361,7 @@
       <c r="M38">
         <v>0</v>
       </c>
-      <c r="O38">
+      <c r="O38" s="1">
         <v>0</v>
       </c>
       <c r="R38" s="1">
@@ -24489,7 +24405,7 @@
       <c r="M39">
         <v>0</v>
       </c>
-      <c r="O39">
+      <c r="O39" s="1">
         <v>0</v>
       </c>
       <c r="R39" s="1">
@@ -24533,7 +24449,7 @@
       <c r="M40">
         <v>0</v>
       </c>
-      <c r="O40">
+      <c r="O40" s="1">
         <v>0</v>
       </c>
       <c r="R40" s="1">
@@ -24577,7 +24493,7 @@
       <c r="M41">
         <v>0</v>
       </c>
-      <c r="O41">
+      <c r="O41" s="1">
         <v>0</v>
       </c>
       <c r="R41" s="1">
@@ -24621,7 +24537,7 @@
       <c r="M42">
         <v>0</v>
       </c>
-      <c r="O42">
+      <c r="O42" s="1">
         <v>0</v>
       </c>
       <c r="R42" s="1">
@@ -24665,7 +24581,7 @@
       <c r="M43">
         <v>0</v>
       </c>
-      <c r="O43">
+      <c r="O43" s="1">
         <v>0</v>
       </c>
       <c r="R43" s="1">
@@ -24709,7 +24625,7 @@
       <c r="M44">
         <v>0</v>
       </c>
-      <c r="O44">
+      <c r="O44" s="1">
         <v>0</v>
       </c>
       <c r="R44" s="1">
@@ -24752,7 +24668,7 @@
       <c r="M45">
         <v>0</v>
       </c>
-      <c r="O45">
+      <c r="O45" s="1">
         <v>0</v>
       </c>
       <c r="R45" s="1">
@@ -24795,7 +24711,7 @@
       <c r="M46">
         <v>0</v>
       </c>
-      <c r="O46">
+      <c r="O46" s="1">
         <v>0</v>
       </c>
       <c r="R46" s="1">
@@ -24838,7 +24754,7 @@
       <c r="M47">
         <v>0</v>
       </c>
-      <c r="O47">
+      <c r="O47" s="1">
         <v>0</v>
       </c>
       <c r="R47" s="1">
@@ -24881,7 +24797,7 @@
       <c r="M48">
         <v>0</v>
       </c>
-      <c r="O48">
+      <c r="O48" s="1">
         <v>0</v>
       </c>
       <c r="R48" s="1">
@@ -24924,7 +24840,7 @@
       <c r="M49">
         <v>0</v>
       </c>
-      <c r="O49">
+      <c r="O49" s="1">
         <v>0</v>
       </c>
       <c r="R49" s="1">
@@ -24967,7 +24883,7 @@
       <c r="M50">
         <v>0</v>
       </c>
-      <c r="O50">
+      <c r="O50" s="1">
         <v>0</v>
       </c>
       <c r="R50" s="1">
@@ -25010,7 +24926,7 @@
       <c r="M51">
         <v>0</v>
       </c>
-      <c r="O51">
+      <c r="O51" s="1">
         <v>0</v>
       </c>
       <c r="R51" s="1">
@@ -25053,7 +24969,7 @@
       <c r="M52">
         <v>0</v>
       </c>
-      <c r="O52">
+      <c r="O52" s="1">
         <v>0</v>
       </c>
       <c r="R52" s="1">
@@ -25096,7 +25012,7 @@
       <c r="M53">
         <v>0</v>
       </c>
-      <c r="O53">
+      <c r="O53" s="1">
         <v>0</v>
       </c>
       <c r="R53" s="1">
@@ -25139,7 +25055,7 @@
       <c r="M54">
         <v>0</v>
       </c>
-      <c r="O54">
+      <c r="O54" s="1">
         <v>0</v>
       </c>
       <c r="R54" s="1">
@@ -25182,7 +25098,7 @@
       <c r="M55">
         <v>0</v>
       </c>
-      <c r="O55">
+      <c r="O55" s="1">
         <v>0</v>
       </c>
       <c r="R55" s="1">
@@ -25225,7 +25141,7 @@
       <c r="M56">
         <v>0</v>
       </c>
-      <c r="O56">
+      <c r="O56" s="1">
         <v>0</v>
       </c>
       <c r="R56" s="1">
@@ -25268,7 +25184,7 @@
       <c r="M57">
         <v>0</v>
       </c>
-      <c r="O57">
+      <c r="O57" s="1">
         <v>0</v>
       </c>
       <c r="R57" s="1">
@@ -25311,7 +25227,7 @@
       <c r="M58">
         <v>0</v>
       </c>
-      <c r="O58">
+      <c r="O58" s="1">
         <v>0</v>
       </c>
       <c r="R58" s="1">
@@ -25354,7 +25270,7 @@
       <c r="M59">
         <v>0</v>
       </c>
-      <c r="O59">
+      <c r="O59" s="1">
         <v>0</v>
       </c>
       <c r="R59" s="1">
@@ -25397,7 +25313,7 @@
       <c r="M60">
         <v>0</v>
       </c>
-      <c r="O60">
+      <c r="O60" s="1">
         <v>0</v>
       </c>
       <c r="R60" s="1">
@@ -25440,7 +25356,7 @@
       <c r="M61">
         <v>0</v>
       </c>
-      <c r="O61">
+      <c r="O61" s="1">
         <v>0</v>
       </c>
       <c r="R61" s="1">
@@ -25483,7 +25399,7 @@
       <c r="M62">
         <v>0</v>
       </c>
-      <c r="O62">
+      <c r="O62" s="1">
         <v>0</v>
       </c>
       <c r="R62" s="1">
@@ -25526,7 +25442,7 @@
       <c r="M63">
         <v>0</v>
       </c>
-      <c r="O63">
+      <c r="O63" s="1">
         <v>0</v>
       </c>
       <c r="R63" s="1">
@@ -25569,7 +25485,7 @@
       <c r="M64">
         <v>0</v>
       </c>
-      <c r="O64">
+      <c r="O64" s="1">
         <v>0</v>
       </c>
       <c r="R64" s="1">
@@ -25612,7 +25528,7 @@
       <c r="M65">
         <v>0</v>
       </c>
-      <c r="O65">
+      <c r="O65" s="1">
         <v>0</v>
       </c>
       <c r="R65" s="1">
@@ -25655,7 +25571,7 @@
       <c r="M66">
         <v>0</v>
       </c>
-      <c r="O66">
+      <c r="O66" s="1">
         <v>0</v>
       </c>
       <c r="R66" s="1">
@@ -25698,7 +25614,7 @@
       <c r="M67">
         <v>0</v>
       </c>
-      <c r="O67">
+      <c r="O67" s="1">
         <v>0</v>
       </c>
       <c r="R67" s="1">
@@ -25741,7 +25657,7 @@
       <c r="M68">
         <v>0</v>
       </c>
-      <c r="O68">
+      <c r="O68" s="1">
         <v>0</v>
       </c>
       <c r="R68" s="1">
@@ -25785,7 +25701,7 @@
       <c r="M69">
         <v>0</v>
       </c>
-      <c r="O69">
+      <c r="O69" s="1">
         <v>0</v>
       </c>
       <c r="R69" s="1">
@@ -25829,7 +25745,7 @@
       <c r="M70">
         <v>0</v>
       </c>
-      <c r="O70">
+      <c r="O70" s="1">
         <v>0</v>
       </c>
       <c r="R70" s="1">
@@ -25869,7 +25785,7 @@
       <c r="M71">
         <v>0</v>
       </c>
-      <c r="O71">
+      <c r="O71" s="1">
         <v>0</v>
       </c>
       <c r="R71" s="1">
@@ -25905,7 +25821,7 @@
       <c r="M72">
         <v>0</v>
       </c>
-      <c r="O72">
+      <c r="O72" s="1">
         <v>0</v>
       </c>
       <c r="R72" s="1">

</xml_diff>